<commit_message>
Implement deferred device addressing (D17) to allow creation of devices without immediate IP assignments
This update amends the device importer to support the creation of new devices whose types define management or loopback interfaces, even when all address cells are left blank. Such rows will raise a `DEVICE_IP_DEFERRED` warning instead of blocking the import, allowing for a two-step process where devices can be created first and addresses added later. Documentation and sample sheets have been updated to reflect this new workflow, ensuring clarity on the deferred addressing process. Tests have been added to validate the new behavior and ensure compliance with the updated requirements.
</commit_message>
<xml_diff>
--- a/samples/2_devices_invalid.xlsx
+++ b/samples/2_devices_invalid.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -436,6 +436,8 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,6 +519,16 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>management_ip6</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>primary address v4</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>primary address v6</t>
         </is>
       </c>
     </row>
@@ -577,6 +589,12 @@
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>192.0.2.30/24</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -635,6 +653,8 @@
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -693,6 +713,8 @@
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -751,6 +773,8 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -809,6 +833,8 @@
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -867,6 +893,8 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -925,6 +953,8 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -983,6 +1013,8 @@
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1041,6 +1073,8 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1099,6 +1133,8 @@
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1153,6 +1189,12 @@
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>192.0.2.51/24</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1211,6 +1253,8 @@
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1269,6 +1313,8 @@
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1327,6 +1373,8 @@
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1385,6 +1433,8 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>